<commit_message>
XGBoosting voi score 0.12485
</commit_message>
<xml_diff>
--- a/Chalenge2/reports/featureEngineering_summary.xlsx
+++ b/Chalenge2/reports/featureEngineering_summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\ml_personalNGroup\Group\chalenge2\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB575B9C-A67D-4BD0-B493-531ACAFDD019}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37FB05FF-9181-4BE5-97FB-44346B85FBDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="31">
   <si>
     <t>Thời gian</t>
   </si>
@@ -110,6 +110,9 @@
   </si>
   <si>
     <t>Đã chuẩn hóa dữ liệu số bằng StandardScaler cho cả train và test.</t>
+  </si>
+  <si>
+    <t>2025-10-27 19:39:16</t>
   </si>
 </sst>
 </file>
@@ -472,11 +475,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.90625" customWidth="1"/>
-    <col min="2" max="2" width="74.26953125" customWidth="1"/>
+    <col min="1" max="1" width="25.6328125" customWidth="1"/>
+    <col min="2" max="2" width="52.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -589,6 +592,83 @@
         <v>29</v>
       </c>
     </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" t="s">
+        <v>22</v>
+      </c>
+      <c r="C17" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>